<commit_message>
Updated Golden question (48)
</commit_message>
<xml_diff>
--- a/kb/Human validated 50 questions.xlsx
+++ b/kb/Human validated 50 questions.xlsx
@@ -571,7 +571,7 @@
     <t>Covington, Henry County has 2 Materials‑category suppliers that could support battery thermal management production for a new Tier 1 company in Georgia.</t>
   </si>
   <si>
-    <t>How many Georgia areas have concentrated Manufacturing Plant facilities but no EV-specific production presence, indicating potential conversion-ready industrial sites?</t>
+    <t>Which Georgia areas have concentrated Manufacturing Plant facilities that already supply the EV chain indirectly but have no dedicated EV production yet,  marking them as prime conversion candidates?</t>
   </si>
   <si>
     <t>There are 100 Georgia areas that currently host Manufacturing Plant facilities but have no EV‑specific production presence, indicating a large pool of potentially conversion‑ready industrial sites.
@@ -1076,7 +1076,7 @@
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="276" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="261.75" customFormat="1" s="1">
       <c r="A2" s="4">
         <v>1</v>
       </c>

</xml_diff>